<commit_message>
feat: add outlier removal, fix minor mistakes
</commit_message>
<xml_diff>
--- a/demo/Results_chocolate/Anova.xlsx
+++ b/demo/Results_chocolate/Anova.xlsx
@@ -483,19 +483,19 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>7.404</v>
+        <v>7.362</v>
       </c>
       <c r="E2" t="n">
-        <v>7.404</v>
+        <v>7.362</v>
       </c>
       <c r="F2" t="n">
-        <v>0.006509247847627415</v>
+        <v>0.006661783100676028</v>
       </c>
       <c r="G2" t="n">
-        <v>0.01459192280707287</v>
+        <v>0.01459665874907309</v>
       </c>
       <c r="H2" t="n">
-        <v>0.2433762519228201</v>
+        <v>0.24341632865181</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -523,19 +523,19 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>448.703</v>
+        <v>438.78</v>
       </c>
       <c r="E3" t="n">
-        <v>448.703</v>
+        <v>438.78</v>
       </c>
       <c r="F3" t="n">
-        <v>1.381480265516726e-99</v>
+        <v>1.995431407933601e-97</v>
       </c>
       <c r="G3" t="n">
-        <v>0.4729646686054539</v>
+        <v>0.4688922610015174</v>
       </c>
       <c r="H3" t="n">
-        <v>1.89463030694645</v>
+        <v>1.879209560274897</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -563,19 +563,19 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>209.305</v>
+        <v>222.403</v>
       </c>
       <c r="E4" t="n">
-        <v>209.305</v>
+        <v>222.403</v>
       </c>
       <c r="F4" t="n">
-        <v>1.947586099985543e-47</v>
+        <v>2.705147253166012e-50</v>
       </c>
       <c r="G4" t="n">
-        <v>0.2950846250907578</v>
+        <v>0.3091493919263612</v>
       </c>
       <c r="H4" t="n">
-        <v>1.294001545594131</v>
+        <v>1.337895280915579</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>

</xml_diff>